<commit_message>
## 2026-10-24 STEAM-DESKTOP-22D / 22F 轨迹补帧与持续打窝## 2026-10-24 STEAM-DESKTOP-22E 入塘与离席表现
</commit_message>
<xml_diff>
--- a/docs/planning/项目开发需求计划表.xlsx
+++ b/docs/planning/项目开发需求计划表.xlsx
@@ -13988,7 +13988,7 @@
       </c>
       <c r="B241" t="inlineStr">
         <is>
-          <t>STEAM-DESKTOP-07A</t>
+          <t>STEAM-DESKTOP-22A</t>
         </is>
       </c>
       <c r="C241" t="inlineStr">
@@ -13998,7 +13998,7 @@
       </c>
       <c r="D241" t="inlineStr">
         <is>
-          <t>桌面宠物主视图与鱼塘入口</t>
+          <t>咬钩读条手账风格</t>
         </is>
       </c>
       <c r="E241" t="inlineStr">
@@ -14008,32 +14008,32 @@
       </c>
       <c r="F241" t="inlineStr">
         <is>
-          <t>v1.0-steam-desktop</t>
+          <t>hotfix</t>
         </is>
       </c>
       <c r="G241" t="inlineStr">
         <is>
-          <t>P0</t>
+          <t>P1</t>
         </is>
       </c>
       <c r="H241" t="inlineStr">
         <is>
-          <t>显示自己的 2D 猫咪、钓鱼状态和鱼塘入口；采用序列帧+状态机，复用已完成桌面壳</t>
+          <t>奶油纸底、暖橙矢量进度与棕色图标；原倒计时保留；Windows视觉待验收</t>
         </is>
       </c>
       <c r="I241" t="inlineStr">
         <is>
-          <t>docs/planning/specs/Steam桌面宠物与多人鱼塘表现层.md</t>
+          <t>docs/planning/specs/Steam桌面端-22鱼塘表现修复与后续迭代.md</t>
         </is>
       </c>
       <c r="J241" t="inlineStr">
         <is>
-          <t>2026-08-13</t>
+          <t>2026-10-24</t>
         </is>
       </c>
       <c r="K241" t="inlineStr">
         <is>
-          <t>2026-08-14</t>
+          <t>2026-10-24</t>
         </is>
       </c>
     </row>
@@ -14045,17 +14045,17 @@
       </c>
       <c r="B242" t="inlineStr">
         <is>
-          <t>STEAM-DESKTOP-07B</t>
+          <t>STEAM-DESKTOP-22B</t>
         </is>
       </c>
       <c r="C242" t="inlineStr">
         <is>
-          <t>功能</t>
+          <t>Bug修复</t>
         </is>
       </c>
       <c r="D242" t="inlineStr">
         <is>
-          <t>2D 鱼塘环境与自己的猫咪</t>
+          <t>鱼线鱼饵水面接触</t>
         </is>
       </c>
       <c r="E242" t="inlineStr">
@@ -14065,32 +14065,32 @@
       </c>
       <c r="F242" t="inlineStr">
         <is>
-          <t>v1.0-steam-desktop</t>
+          <t>hotfix</t>
         </is>
       </c>
       <c r="G242" t="inlineStr">
         <is>
-          <t>P0</t>
+          <t>P1</t>
         </is>
       </c>
       <c r="H242" t="inlineStr">
         <is>
-          <t>显示池塘环境、钓位、自己的宠物和钓鱼表现</t>
+          <t>按座位前沿校正浮漂／鱼及竿尖固定的鱼线长度；收杆渐退；6组数学测试通过，Windows视觉待验收</t>
         </is>
       </c>
       <c r="I242" t="inlineStr">
         <is>
-          <t>docs/planning/specs/Steam桌面宠物与多人鱼塘表现层.md</t>
+          <t>docs/planning/specs/Steam桌面端-22鱼塘表现修复与后续迭代.md</t>
         </is>
       </c>
       <c r="J242" t="inlineStr">
         <is>
-          <t>2026-08-13</t>
+          <t>2026-10-24</t>
         </is>
       </c>
       <c r="K242" t="inlineStr">
         <is>
-          <t>2026-08-14</t>
+          <t>2026-10-24</t>
         </is>
       </c>
     </row>
@@ -14102,17 +14102,17 @@
       </c>
       <c r="B243" t="inlineStr">
         <is>
-          <t>STEAM-DESKTOP-07C</t>
+          <t>STEAM-DESKTOP-22C</t>
         </is>
       </c>
       <c r="C243" t="inlineStr">
         <is>
-          <t>功能</t>
+          <t>Bug修复</t>
         </is>
       </c>
       <c r="D243" t="inlineStr">
         <is>
-          <t>同塘玩家宠物与状态同步</t>
+          <t>Overlay聊天展开</t>
         </is>
       </c>
       <c r="E243" t="inlineStr">
@@ -14122,7 +14122,7 @@
       </c>
       <c r="F243" t="inlineStr">
         <is>
-          <t>v1.0-steam-desktop</t>
+          <t>hotfix</t>
         </is>
       </c>
       <c r="G243" t="inlineStr">
@@ -14132,22 +14132,22 @@
       </c>
       <c r="H243" t="inlineStr">
         <is>
-          <t>在 Overlay 渲染 pond_user_joined/left/updated；128×128 统一序列帧；fishingPhase→petVisualState；IPC 不传图、不新开协议</t>
+          <t>折叠栏与开关预览按下展开，命中缓存失效；原生测试加入真实输入路由，Windows点击待验收</t>
         </is>
       </c>
       <c r="I243" t="inlineStr">
         <is>
-          <t>docs/planning/specs/Steam桌面宠物与多人鱼塘表现层.md</t>
+          <t>docs/planning/specs/Steam桌面端-22鱼塘表现修复与后续迭代.md</t>
         </is>
       </c>
       <c r="J243" t="inlineStr">
         <is>
-          <t>2026-08-13</t>
+          <t>2026-10-24</t>
         </is>
       </c>
       <c r="K243" t="inlineStr">
         <is>
-          <t>2026-08-15</t>
+          <t>2026-10-24</t>
         </is>
       </c>
     </row>
@@ -14159,7 +14159,7 @@
       </c>
       <c r="B244" t="inlineStr">
         <is>
-          <t>STEAM-DESKTOP-07D</t>
+          <t>STEAM-DESKTOP-22D</t>
         </is>
       </c>
       <c r="C244" t="inlineStr">
@@ -14169,7 +14169,7 @@
       </c>
       <c r="D244" t="inlineStr">
         <is>
-          <t>桌面宠物右键菜单</t>
+          <t>Overlay动画补帧</t>
         </is>
       </c>
       <c r="E244" t="inlineStr">
@@ -14179,32 +14179,32 @@
       </c>
       <c r="F244" t="inlineStr">
         <is>
-          <t>v1.0-steam-desktop</t>
+          <t>后续迭代</t>
         </is>
       </c>
       <c r="G244" t="inlineStr">
         <is>
-          <t>P0</t>
+          <t>P2</t>
         </is>
       </c>
       <c r="H244" t="inlineStr">
         <is>
-          <t>在产品窗口/宠物区域提供鱼塘、好友、背包、图鉴、设置、托盘和退出入口</t>
+          <t>抛竿13、收杆/空军16、打窝18个分层轨迹采样；总时长不变、复用PNG缓存；Windows原生待验收</t>
         </is>
       </c>
       <c r="I244" t="inlineStr">
         <is>
-          <t>docs/planning/specs/Steam桌面宠物与多人鱼塘表现层.md</t>
+          <t>docs/planning/specs/Steam桌面端-22鱼塘表现修复与后续迭代.md</t>
         </is>
       </c>
       <c r="J244" t="inlineStr">
         <is>
-          <t>2026-08-13</t>
+          <t>2026-10-24</t>
         </is>
       </c>
       <c r="K244" t="inlineStr">
         <is>
-          <t>2026-08-16</t>
+          <t>2026-10-24</t>
         </is>
       </c>
     </row>
@@ -14216,7 +14216,7 @@
       </c>
       <c r="B245" t="inlineStr">
         <is>
-          <t>STEAM-DESKTOP-07E</t>
+          <t>STEAM-DESKTOP-22E</t>
         </is>
       </c>
       <c r="C245" t="inlineStr">
@@ -14226,7 +14226,7 @@
       </c>
       <c r="D245" t="inlineStr">
         <is>
-          <t>桌面宠物主窗口功能页签</t>
+          <t>入塘离席猫咪位置与站起时序</t>
         </is>
       </c>
       <c r="E245" t="inlineStr">
@@ -14236,32 +14236,32 @@
       </c>
       <c r="F245" t="inlineStr">
         <is>
-          <t>v1.0-steam-desktop</t>
+          <t>hotfix</t>
         </is>
       </c>
       <c r="G245" t="inlineStr">
         <is>
-          <t>P0</t>
+          <t>P2</t>
         </is>
       </c>
       <c r="H245" t="inlineStr">
         <is>
-          <t>好友/聊天、背包、图鉴、设置为主窗口页签；Overlay 菜单切页且主窗口高于 Overlay；不用功能弹窗</t>
+          <t>脚底锚点统一；到位后坐下、站起尾帧结束再平滑离席；重复快照与重入保护；Windows视觉待验收</t>
         </is>
       </c>
       <c r="I245" t="inlineStr">
         <is>
-          <t>docs/planning/specs/Steam桌面端Web功能对齐设计.md</t>
+          <t>docs/planning/specs/Steam桌面端-22鱼塘表现修复与后续迭代.md</t>
         </is>
       </c>
       <c r="J245" t="inlineStr">
         <is>
-          <t>2026-08-13</t>
+          <t>2026-10-24</t>
         </is>
       </c>
       <c r="K245" t="inlineStr">
         <is>
-          <t>2026-08-17</t>
+          <t>2026-10-24</t>
         </is>
       </c>
     </row>
@@ -14273,7 +14273,7 @@
       </c>
       <c r="B246" t="inlineStr">
         <is>
-          <t>STEAM-DESKTOP-07F</t>
+          <t>STEAM-DESKTOP-22F</t>
         </is>
       </c>
       <c r="C246" t="inlineStr">
@@ -14283,7 +14283,7 @@
       </c>
       <c r="D246" t="inlineStr">
         <is>
-          <t>桌面宠物主流程与恢复验收</t>
+          <t>打窝循环动画</t>
         </is>
       </c>
       <c r="E246" t="inlineStr">
@@ -14293,44 +14293,44 @@
       </c>
       <c r="F246" t="inlineStr">
         <is>
-          <t>v1.0-steam-desktop</t>
+          <t>后续迭代</t>
         </is>
       </c>
       <c r="G246" t="inlineStr">
         <is>
-          <t>P0</t>
+          <t>P2</t>
         </is>
       </c>
       <c r="H246" t="inlineStr">
         <is>
-          <t>串联登录、进塘、挂机、通知、托盘、收鱼、断线恢复并完成 Windows 验收</t>
+          <t>100ms起手/720ms循环/280ms收尾，直到groundbaiting真实退出；网络更新与中断保护；Windows原生待验收</t>
         </is>
       </c>
       <c r="I246" t="inlineStr">
         <is>
-          <t>docs/planning/specs/Steam桌面宠物与多人鱼塘表现层.md</t>
+          <t>docs/planning/specs/Steam桌面端-22鱼塘表现修复与后续迭代.md</t>
         </is>
       </c>
       <c r="J246" t="inlineStr">
         <is>
-          <t>2026-08-13</t>
+          <t>2026-10-24</t>
         </is>
       </c>
       <c r="K246" t="inlineStr">
         <is>
-          <t>2026-08-17</t>
+          <t>2026-10-24</t>
         </is>
       </c>
     </row>
     <row r="247">
       <c r="A247" t="inlineStr">
         <is>
-          <t>已实现</t>
+          <t>已确认</t>
         </is>
       </c>
       <c r="B247" t="inlineStr">
         <is>
-          <t>STEAM-DESKTOP-07G</t>
+          <t>STEAM-DESKTOP-22G</t>
         </is>
       </c>
       <c r="C247" t="inlineStr">
@@ -14340,7 +14340,7 @@
       </c>
       <c r="D247" t="inlineStr">
         <is>
-          <t>原生桌面宠物 Overlay</t>
+          <t>Overlay背景场景美术迭代</t>
         </is>
       </c>
       <c r="E247" t="inlineStr">
@@ -14350,44 +14350,39 @@
       </c>
       <c r="F247" t="inlineStr">
         <is>
-          <t>v1.0-steam-desktop</t>
+          <t>后续迭代</t>
         </is>
       </c>
       <c r="G247" t="inlineStr">
         <is>
-          <t>P1</t>
+          <t>P2</t>
         </is>
       </c>
       <c r="H247" t="inlineStr">
         <is>
-          <t>独立 WPF/Win32 Overlay；不启动第二个 Unity Player；通过 Named Pipe 接收状态并发送命令</t>
+          <t>仅记录：岸线、水面、钓位层次与风格优化，先预览后替换</t>
         </is>
       </c>
       <c r="I247" t="inlineStr">
         <is>
-          <t>docs/planning/specs/Steam原生桌面宠物Overlay.md</t>
+          <t>docs/planning/specs/Steam桌面端-22鱼塘表现修复与后续迭代.md</t>
         </is>
       </c>
       <c r="J247" t="inlineStr">
         <is>
-          <t>2026-08-14</t>
-        </is>
-      </c>
-      <c r="K247" t="inlineStr">
-        <is>
-          <t>2026-08-17</t>
+          <t>2026-10-24</t>
         </is>
       </c>
     </row>
     <row r="248">
       <c r="A248" t="inlineStr">
         <is>
-          <t>已实现</t>
+          <t>已确认</t>
         </is>
       </c>
       <c r="B248" t="inlineStr">
         <is>
-          <t>STEAM-DESKTOP-08A</t>
+          <t>STEAM-DESKTOP-22H</t>
         </is>
       </c>
       <c r="C248" t="inlineStr">
@@ -14397,7 +14392,7 @@
       </c>
       <c r="D248" t="inlineStr">
         <is>
-          <t>世界地图与鱼塘选择</t>
+          <t>钓鱼过程特效</t>
         </is>
       </c>
       <c r="E248" t="inlineStr">
@@ -14407,44 +14402,39 @@
       </c>
       <c r="F248" t="inlineStr">
         <is>
-          <t>v1.0-steam-desktop</t>
+          <t>后续迭代</t>
         </is>
       </c>
       <c r="G248" t="inlineStr">
         <is>
-          <t>P0</t>
+          <t>P2</t>
         </is>
       </c>
       <c r="H248" t="inlineStr">
         <is>
-          <t>主窗口超大地图 Image：拖动/滚轮缩放/边界；pondId 坐标绑定；点击进塘并显示 Overlay</t>
+          <t>仅记录：入水、波纹、咬钩、挣扎、收杆、脱钩反馈</t>
         </is>
       </c>
       <c r="I248" t="inlineStr">
         <is>
-          <t>docs/planning/specs/Steam桌面端-08A世界地图与鱼塘选择.md</t>
+          <t>docs/planning/specs/Steam桌面端-22鱼塘表现修复与后续迭代.md</t>
         </is>
       </c>
       <c r="J248" t="inlineStr">
         <is>
-          <t>2026-08-17</t>
-        </is>
-      </c>
-      <c r="K248" t="inlineStr">
-        <is>
-          <t>2026-08-17</t>
+          <t>2026-10-24</t>
         </is>
       </c>
     </row>
     <row r="249">
       <c r="A249" t="inlineStr">
         <is>
-          <t>已实现</t>
+          <t>已确认</t>
         </is>
       </c>
       <c r="B249" t="inlineStr">
         <is>
-          <t>STEAM-DESKTOP-08B</t>
+          <t>STEAM-DESKTOP-22I</t>
         </is>
       </c>
       <c r="C249" t="inlineStr">
@@ -14454,7 +14444,7 @@
       </c>
       <c r="D249" t="inlineStr">
         <is>
-          <t>商店与装备</t>
+          <t>钓鱼与UI音效迭代</t>
         </is>
       </c>
       <c r="E249" t="inlineStr">
@@ -14464,44 +14454,39 @@
       </c>
       <c r="F249" t="inlineStr">
         <is>
-          <t>v1.0-steam-desktop</t>
+          <t>后续迭代</t>
         </is>
       </c>
       <c r="G249" t="inlineStr">
         <is>
-          <t>P0</t>
+          <t>P2</t>
         </is>
       </c>
       <c r="H249" t="inlineStr">
         <is>
-          <t>PanelShop：鱼饵/渔具购买与装备；金币库存以服务端为准；Overlay 只 menu_shop 切页</t>
+          <t>仅记录：音色、音量、触发时机与并发控制</t>
         </is>
       </c>
       <c r="I249" t="inlineStr">
         <is>
-          <t>docs/planning/specs/Steam桌面端-08B商店与装备.md</t>
+          <t>docs/planning/specs/Steam桌面端-22鱼塘表现修复与后续迭代.md</t>
         </is>
       </c>
       <c r="J249" t="inlineStr">
         <is>
-          <t>2026-08-17</t>
-        </is>
-      </c>
-      <c r="K249" t="inlineStr">
-        <is>
-          <t>2026-08-18</t>
+          <t>2026-10-24</t>
         </is>
       </c>
     </row>
     <row r="250">
       <c r="A250" t="inlineStr">
         <is>
-          <t>已实现</t>
+          <t>已确认</t>
         </is>
       </c>
       <c r="B250" t="inlineStr">
         <is>
-          <t>STEAM-DESKTOP-08C</t>
+          <t>STEAM-DESKTOP-22J</t>
         </is>
       </c>
       <c r="C250" t="inlineStr">
@@ -14511,7 +14496,7 @@
       </c>
       <c r="D250" t="inlineStr">
         <is>
-          <t>动态墙与好友动态</t>
+          <t>世界地图迭代</t>
         </is>
       </c>
       <c r="E250" t="inlineStr">
@@ -14521,32 +14506,27 @@
       </c>
       <c r="F250" t="inlineStr">
         <is>
-          <t>v1.0-steam-desktop</t>
+          <t>后续迭代</t>
         </is>
       </c>
       <c r="G250" t="inlineStr">
         <is>
-          <t>P1</t>
+          <t>P2</t>
         </is>
       </c>
       <c r="H250" t="inlineStr">
         <is>
-          <t>PanelSocialFeed：公共/好友动态、分页加载、动态卡片 Prefab、点赞、评论、删除评论；不塞进 PanelSocial</t>
+          <t>仅记录：信息层级、标识、筛选详情与进入路径；先交互预览</t>
         </is>
       </c>
       <c r="I250" t="inlineStr">
         <is>
-          <t>docs/planning/specs/Steam桌面端-08C动态墙与好友动态.md</t>
+          <t>docs/planning/specs/Steam桌面端-22鱼塘表现修复与后续迭代.md</t>
         </is>
       </c>
       <c r="J250" t="inlineStr">
         <is>
-          <t>2026-08-17</t>
-        </is>
-      </c>
-      <c r="K250" t="inlineStr">
-        <is>
-          <t>2026-08-19</t>
+          <t>2026-10-24</t>
         </is>
       </c>
     </row>
@@ -14558,7 +14538,7 @@
       </c>
       <c r="B251" t="inlineStr">
         <is>
-          <t>STEAM-DESKTOP-08D</t>
+          <t>STEAM-DESKTOP-07A</t>
         </is>
       </c>
       <c r="C251" t="inlineStr">
@@ -14568,7 +14548,7 @@
       </c>
       <c r="D251" t="inlineStr">
         <is>
-          <t>排行榜</t>
+          <t>桌面宠物主视图与鱼塘入口</t>
         </is>
       </c>
       <c r="E251" t="inlineStr">
@@ -14583,27 +14563,27 @@
       </c>
       <c r="G251" t="inlineStr">
         <is>
-          <t>P1</t>
+          <t>P0</t>
         </is>
       </c>
       <c r="H251" t="inlineStr">
         <is>
-          <t>PanelLeaderboard：日/周/鱼塘/稀有四榜；Top3 固定 Image 领奖台；4 名起纵向滚动；分数以服务端为准</t>
+          <t>显示自己的 2D 猫咪、钓鱼状态和鱼塘入口；采用序列帧+状态机，复用已完成桌面壳</t>
         </is>
       </c>
       <c r="I251" t="inlineStr">
         <is>
-          <t>docs/planning/specs/Steam桌面端-08D排行榜.md</t>
+          <t>docs/planning/specs/Steam桌面宠物与多人鱼塘表现层.md</t>
         </is>
       </c>
       <c r="J251" t="inlineStr">
         <is>
-          <t>2026-08-17</t>
+          <t>2026-08-13</t>
         </is>
       </c>
       <c r="K251" t="inlineStr">
         <is>
-          <t>2026-08-20</t>
+          <t>2026-08-14</t>
         </is>
       </c>
     </row>
@@ -14615,7 +14595,7 @@
       </c>
       <c r="B252" t="inlineStr">
         <is>
-          <t>STEAM-DESKTOP-08E</t>
+          <t>STEAM-DESKTOP-07B</t>
         </is>
       </c>
       <c r="C252" t="inlineStr">
@@ -14625,7 +14605,7 @@
       </c>
       <c r="D252" t="inlineStr">
         <is>
-          <t>个人中心与资料编辑</t>
+          <t>2D 鱼塘环境与自己的猫咪</t>
         </is>
       </c>
       <c r="E252" t="inlineStr">
@@ -14640,27 +14620,27 @@
       </c>
       <c r="G252" t="inlineStr">
         <is>
-          <t>P1</t>
+          <t>P0</t>
         </is>
       </c>
       <c r="H252" t="inlineStr">
         <is>
-          <t>PanelProfile/Edit：昵称头像展示鱼获；不改 SteamID、不迁移旧档</t>
+          <t>显示池塘环境、钓位、自己的宠物和钓鱼表现</t>
         </is>
       </c>
       <c r="I252" t="inlineStr">
         <is>
-          <t>docs/planning/specs/Steam桌面端-08E个人中心与资料编辑.md</t>
+          <t>docs/planning/specs/Steam桌面宠物与多人鱼塘表现层.md</t>
         </is>
       </c>
       <c r="J252" t="inlineStr">
         <is>
-          <t>2026-08-17</t>
+          <t>2026-08-13</t>
         </is>
       </c>
       <c r="K252" t="inlineStr">
         <is>
-          <t>2026-08-18</t>
+          <t>2026-08-14</t>
         </is>
       </c>
     </row>
@@ -14672,7 +14652,7 @@
       </c>
       <c r="B253" t="inlineStr">
         <is>
-          <t>STEAM-DESKTOP-08F</t>
+          <t>STEAM-DESKTOP-07C</t>
         </is>
       </c>
       <c r="C253" t="inlineStr">
@@ -14682,7 +14662,7 @@
       </c>
       <c r="D253" t="inlineStr">
         <is>
-          <t>好友列表与申请 Prefab</t>
+          <t>同塘玩家宠物与状态同步</t>
         </is>
       </c>
       <c r="E253" t="inlineStr">
@@ -14702,22 +14682,22 @@
       </c>
       <c r="H253" t="inlineStr">
         <is>
-          <t>独立 PanelFriends；修复接受/拒绝重叠不可点；不与 PanelSocial 双开好友 UI</t>
+          <t>在 Overlay 渲染 pond_user_joined/left/updated；128×128 统一序列帧；fishingPhase→petVisualState；IPC 不传图、不新开协议</t>
         </is>
       </c>
       <c r="I253" t="inlineStr">
         <is>
-          <t>docs/planning/specs/Steam桌面端-08F好友列表与申请Prefab.md</t>
+          <t>docs/planning/specs/Steam桌面宠物与多人鱼塘表现层.md</t>
         </is>
       </c>
       <c r="J253" t="inlineStr">
         <is>
-          <t>2026-08-17</t>
+          <t>2026-08-13</t>
         </is>
       </c>
       <c r="K253" t="inlineStr">
         <is>
-          <t>2026-08-17</t>
+          <t>2026-08-15</t>
         </is>
       </c>
     </row>
@@ -14729,7 +14709,7 @@
       </c>
       <c r="B254" t="inlineStr">
         <is>
-          <t>STEAM-DESKTOP-08G</t>
+          <t>STEAM-DESKTOP-07D</t>
         </is>
       </c>
       <c r="C254" t="inlineStr">
@@ -14739,7 +14719,7 @@
       </c>
       <c r="D254" t="inlineStr">
         <is>
-          <t>Overlay 钓鱼操作栏</t>
+          <t>桌面宠物右键菜单</t>
         </is>
       </c>
       <c r="E254" t="inlineStr">
@@ -14759,22 +14739,22 @@
       </c>
       <c r="H254" t="inlineStr">
         <is>
-          <t>Overlay 底部选钓位/开始/收杆/领鱼获；Pipe 发命令；Unity/Node 保留权威</t>
+          <t>在产品窗口/宠物区域提供鱼塘、好友、背包、图鉴、设置、托盘和退出入口</t>
         </is>
       </c>
       <c r="I254" t="inlineStr">
         <is>
-          <t>docs/planning/specs/Steam桌面端-08GOverlay钓鱼操作栏.md</t>
+          <t>docs/planning/specs/Steam桌面宠物与多人鱼塘表现层.md</t>
         </is>
       </c>
       <c r="J254" t="inlineStr">
         <is>
-          <t>2026-08-17</t>
+          <t>2026-08-13</t>
         </is>
       </c>
       <c r="K254" t="inlineStr">
         <is>
-          <t>2026-08-17</t>
+          <t>2026-08-16</t>
         </is>
       </c>
     </row>
@@ -14786,17 +14766,17 @@
       </c>
       <c r="B255" t="inlineStr">
         <is>
-          <t>STEAM-DESKTOP-08H</t>
+          <t>STEAM-DESKTOP-07E</t>
         </is>
       </c>
       <c r="C255" t="inlineStr">
         <is>
-          <t>工程</t>
+          <t>功能</t>
         </is>
       </c>
       <c r="D255" t="inlineStr">
         <is>
-          <t>全量 UI 预制体化与动态内容组件</t>
+          <t>桌面宠物主窗口功能页签</t>
         </is>
       </c>
       <c r="E255" t="inlineStr">
@@ -14816,17 +14796,17 @@
       </c>
       <c r="H255" t="inlineStr">
         <is>
-          <t>壳层、功能页、列表行和 Grid item 全部使用合法 Prefab；运行时代码只绑定数据和事件</t>
+          <t>好友/聊天、背包、图鉴、设置为主窗口页签；Overlay 菜单切页且主窗口高于 Overlay；不用功能弹窗</t>
         </is>
       </c>
       <c r="I255" t="inlineStr">
         <is>
-          <t>docs/planning/specs/Steam桌面端-08H全量UI预制体化.md</t>
+          <t>docs/planning/specs/Steam桌面端Web功能对齐设计.md</t>
         </is>
       </c>
       <c r="J255" t="inlineStr">
         <is>
-          <t>2026-08-17</t>
+          <t>2026-08-13</t>
         </is>
       </c>
       <c r="K255" t="inlineStr">
@@ -14843,17 +14823,17 @@
       </c>
       <c r="B256" t="inlineStr">
         <is>
-          <t>STEAM-DESKTOP-08I</t>
+          <t>STEAM-DESKTOP-07F</t>
         </is>
       </c>
       <c r="C256" t="inlineStr">
         <is>
-          <t>Bug修复</t>
+          <t>功能</t>
         </is>
       </c>
       <c r="D256" t="inlineStr">
         <is>
-          <t>鱼塘退出与跨塘切换优化</t>
+          <t>桌面宠物主流程与恢复验收</t>
         </is>
       </c>
       <c r="E256" t="inlineStr">
@@ -14873,22 +14853,22 @@
       </c>
       <c r="H256" t="inlineStr">
         <is>
-          <t>Overlay 点击钓位直接入座；新增离席/退出鱼塘；收杆领鱼离席后跨塘切换；修复隐藏主窗口时 5 FPS 导致的 ACK 延迟，增加 ACK 优先队列、持久状态序号、重复状态丢弃及三段链路时间戳验收</t>
+          <t>串联登录、进塘、挂机、通知、托盘、收鱼、断线恢复并完成 Windows 验收</t>
         </is>
       </c>
       <c r="I256" t="inlineStr">
         <is>
-          <t>docs/planning/specs/Steam桌面端-08I鱼塘退出与跨塘切换优化.md</t>
+          <t>docs/planning/specs/Steam桌面宠物与多人鱼塘表现层.md</t>
         </is>
       </c>
       <c r="J256" t="inlineStr">
         <is>
-          <t>2026-08-18</t>
+          <t>2026-08-13</t>
         </is>
       </c>
       <c r="K256" t="inlineStr">
         <is>
-          <t>2026-08-18</t>
+          <t>2026-08-17</t>
         </is>
       </c>
     </row>
@@ -14900,7 +14880,7 @@
       </c>
       <c r="B257" t="inlineStr">
         <is>
-          <t>STEAM-DESKTOP-22A</t>
+          <t>STEAM-DESKTOP-07G</t>
         </is>
       </c>
       <c r="C257" t="inlineStr">
@@ -14910,7 +14890,7 @@
       </c>
       <c r="D257" t="inlineStr">
         <is>
-          <t>咬钩读条手账风格</t>
+          <t>原生桌面宠物 Overlay</t>
         </is>
       </c>
       <c r="E257" t="inlineStr">
@@ -14920,7 +14900,7 @@
       </c>
       <c r="F257" t="inlineStr">
         <is>
-          <t>hotfix</t>
+          <t>v1.0-steam-desktop</t>
         </is>
       </c>
       <c r="G257" t="inlineStr">
@@ -14930,22 +14910,22 @@
       </c>
       <c r="H257" t="inlineStr">
         <is>
-          <t>奶油纸底、暖橙矢量进度与棕色图标；原倒计时保留；Windows视觉待验收</t>
+          <t>独立 WPF/Win32 Overlay；不启动第二个 Unity Player；通过 Named Pipe 接收状态并发送命令</t>
         </is>
       </c>
       <c r="I257" t="inlineStr">
         <is>
-          <t>docs/planning/specs/Steam桌面端-22鱼塘表现修复与后续迭代.md</t>
+          <t>docs/planning/specs/Steam原生桌面宠物Overlay.md</t>
         </is>
       </c>
       <c r="J257" t="inlineStr">
         <is>
-          <t>2026-10-24</t>
+          <t>2026-08-14</t>
         </is>
       </c>
       <c r="K257" t="inlineStr">
         <is>
-          <t>2026-10-24</t>
+          <t>2026-08-17</t>
         </is>
       </c>
     </row>
@@ -14957,17 +14937,17 @@
       </c>
       <c r="B258" t="inlineStr">
         <is>
-          <t>STEAM-DESKTOP-22B</t>
+          <t>STEAM-DESKTOP-08A</t>
         </is>
       </c>
       <c r="C258" t="inlineStr">
         <is>
-          <t>Bug修复</t>
+          <t>功能</t>
         </is>
       </c>
       <c r="D258" t="inlineStr">
         <is>
-          <t>鱼线鱼饵水面接触</t>
+          <t>世界地图与鱼塘选择</t>
         </is>
       </c>
       <c r="E258" t="inlineStr">
@@ -14977,32 +14957,32 @@
       </c>
       <c r="F258" t="inlineStr">
         <is>
-          <t>hotfix</t>
+          <t>v1.0-steam-desktop</t>
         </is>
       </c>
       <c r="G258" t="inlineStr">
         <is>
-          <t>P1</t>
+          <t>P0</t>
         </is>
       </c>
       <c r="H258" t="inlineStr">
         <is>
-          <t>按座位前沿校正浮漂／鱼及竿尖固定的鱼线长度；收杆渐退；6组数学测试通过，Windows视觉待验收</t>
+          <t>主窗口超大地图 Image：拖动/滚轮缩放/边界；pondId 坐标绑定；点击进塘并显示 Overlay</t>
         </is>
       </c>
       <c r="I258" t="inlineStr">
         <is>
-          <t>docs/planning/specs/Steam桌面端-22鱼塘表现修复与后续迭代.md</t>
+          <t>docs/planning/specs/Steam桌面端-08A世界地图与鱼塘选择.md</t>
         </is>
       </c>
       <c r="J258" t="inlineStr">
         <is>
-          <t>2026-10-24</t>
+          <t>2026-08-17</t>
         </is>
       </c>
       <c r="K258" t="inlineStr">
         <is>
-          <t>2026-10-24</t>
+          <t>2026-08-17</t>
         </is>
       </c>
     </row>
@@ -15014,17 +14994,17 @@
       </c>
       <c r="B259" t="inlineStr">
         <is>
-          <t>STEAM-DESKTOP-22C</t>
+          <t>STEAM-DESKTOP-08B</t>
         </is>
       </c>
       <c r="C259" t="inlineStr">
         <is>
-          <t>Bug修复</t>
+          <t>功能</t>
         </is>
       </c>
       <c r="D259" t="inlineStr">
         <is>
-          <t>Overlay聊天展开</t>
+          <t>商店与装备</t>
         </is>
       </c>
       <c r="E259" t="inlineStr">
@@ -15034,7 +15014,7 @@
       </c>
       <c r="F259" t="inlineStr">
         <is>
-          <t>hotfix</t>
+          <t>v1.0-steam-desktop</t>
         </is>
       </c>
       <c r="G259" t="inlineStr">
@@ -15044,34 +15024,34 @@
       </c>
       <c r="H259" t="inlineStr">
         <is>
-          <t>折叠栏与开关预览按下展开，命中缓存失效；原生测试加入真实输入路由，Windows点击待验收</t>
+          <t>PanelShop：鱼饵/渔具购买与装备；金币库存以服务端为准；Overlay 只 menu_shop 切页</t>
         </is>
       </c>
       <c r="I259" t="inlineStr">
         <is>
-          <t>docs/planning/specs/Steam桌面端-22鱼塘表现修复与后续迭代.md</t>
+          <t>docs/planning/specs/Steam桌面端-08B商店与装备.md</t>
         </is>
       </c>
       <c r="J259" t="inlineStr">
         <is>
-          <t>2026-10-24</t>
+          <t>2026-08-17</t>
         </is>
       </c>
       <c r="K259" t="inlineStr">
         <is>
-          <t>2026-10-24</t>
+          <t>2026-08-18</t>
         </is>
       </c>
     </row>
     <row r="260">
       <c r="A260" t="inlineStr">
         <is>
-          <t>已确认</t>
+          <t>已实现</t>
         </is>
       </c>
       <c r="B260" t="inlineStr">
         <is>
-          <t>STEAM-DESKTOP-22D</t>
+          <t>STEAM-DESKTOP-08C</t>
         </is>
       </c>
       <c r="C260" t="inlineStr">
@@ -15081,7 +15061,7 @@
       </c>
       <c r="D260" t="inlineStr">
         <is>
-          <t>Overlay动画补帧</t>
+          <t>动态墙与好友动态</t>
         </is>
       </c>
       <c r="E260" t="inlineStr">
@@ -15091,40 +15071,44 @@
       </c>
       <c r="F260" t="inlineStr">
         <is>
-          <t>后续迭代</t>
+          <t>v1.0-steam-desktop</t>
         </is>
       </c>
       <c r="G260" t="inlineStr">
         <is>
-          <t>P2</t>
+          <t>P1</t>
         </is>
       </c>
       <c r="H260" t="inlineStr">
         <is>
-          <t>仅记录：补关键动作中间帧，控制内存／解码成本</t>
+          <t>PanelSocialFeed：公共/好友动态、分页加载、动态卡片 Prefab、点赞、评论、删除评论；不塞进 PanelSocial</t>
         </is>
       </c>
       <c r="I260" t="inlineStr">
         <is>
-          <t>docs/planning/specs/Steam桌面端-22鱼塘表现修复与后续迭代.md</t>
+          <t>docs/planning/specs/Steam桌面端-08C动态墙与好友动态.md</t>
         </is>
       </c>
       <c r="J260" t="inlineStr">
         <is>
-          <t>2026-10-24</t>
-        </is>
-      </c>
-      <c r="K260" t="inlineStr"/>
+          <t>2026-08-17</t>
+        </is>
+      </c>
+      <c r="K260" t="inlineStr">
+        <is>
+          <t>2026-08-19</t>
+        </is>
+      </c>
     </row>
     <row r="261">
       <c r="A261" t="inlineStr">
         <is>
-          <t>已确认</t>
+          <t>已实现</t>
         </is>
       </c>
       <c r="B261" t="inlineStr">
         <is>
-          <t>STEAM-DESKTOP-22E</t>
+          <t>STEAM-DESKTOP-08D</t>
         </is>
       </c>
       <c r="C261" t="inlineStr">
@@ -15134,7 +15118,7 @@
       </c>
       <c r="D261" t="inlineStr">
         <is>
-          <t>入塘离席猫咪位置与站起时序</t>
+          <t>排行榜</t>
         </is>
       </c>
       <c r="E261" t="inlineStr">
@@ -15144,40 +15128,44 @@
       </c>
       <c r="F261" t="inlineStr">
         <is>
-          <t>后续迭代</t>
+          <t>v1.0-steam-desktop</t>
         </is>
       </c>
       <c r="G261" t="inlineStr">
         <is>
-          <t>P2</t>
+          <t>P1</t>
         </is>
       </c>
       <c r="H261" t="inlineStr">
         <is>
-          <t>仅记录：脚底与钓位对齐，站起结束后再离开</t>
+          <t>PanelLeaderboard：日/周/鱼塘/稀有四榜；Top3 固定 Image 领奖台；4 名起纵向滚动；分数以服务端为准</t>
         </is>
       </c>
       <c r="I261" t="inlineStr">
         <is>
-          <t>docs/planning/specs/Steam桌面端-22鱼塘表现修复与后续迭代.md</t>
+          <t>docs/planning/specs/Steam桌面端-08D排行榜.md</t>
         </is>
       </c>
       <c r="J261" t="inlineStr">
         <is>
-          <t>2026-10-24</t>
-        </is>
-      </c>
-      <c r="K261" t="inlineStr"/>
+          <t>2026-08-17</t>
+        </is>
+      </c>
+      <c r="K261" t="inlineStr">
+        <is>
+          <t>2026-08-20</t>
+        </is>
+      </c>
     </row>
     <row r="262">
       <c r="A262" t="inlineStr">
         <is>
-          <t>已确认</t>
+          <t>已实现</t>
         </is>
       </c>
       <c r="B262" t="inlineStr">
         <is>
-          <t>STEAM-DESKTOP-22F</t>
+          <t>STEAM-DESKTOP-08E</t>
         </is>
       </c>
       <c r="C262" t="inlineStr">
@@ -15187,7 +15175,7 @@
       </c>
       <c r="D262" t="inlineStr">
         <is>
-          <t>打窝循环动画</t>
+          <t>个人中心与资料编辑</t>
         </is>
       </c>
       <c r="E262" t="inlineStr">
@@ -15197,40 +15185,44 @@
       </c>
       <c r="F262" t="inlineStr">
         <is>
-          <t>后续迭代</t>
+          <t>v1.0-steam-desktop</t>
         </is>
       </c>
       <c r="G262" t="inlineStr">
         <is>
-          <t>P2</t>
+          <t>P1</t>
         </is>
       </c>
       <c r="H262" t="inlineStr">
         <is>
-          <t>仅记录：起手、循环、收尾匹配服务器打窝时长</t>
+          <t>PanelProfile/Edit：昵称头像展示鱼获；不改 SteamID、不迁移旧档</t>
         </is>
       </c>
       <c r="I262" t="inlineStr">
         <is>
-          <t>docs/planning/specs/Steam桌面端-22鱼塘表现修复与后续迭代.md</t>
+          <t>docs/planning/specs/Steam桌面端-08E个人中心与资料编辑.md</t>
         </is>
       </c>
       <c r="J262" t="inlineStr">
         <is>
-          <t>2026-10-24</t>
-        </is>
-      </c>
-      <c r="K262" t="inlineStr"/>
+          <t>2026-08-17</t>
+        </is>
+      </c>
+      <c r="K262" t="inlineStr">
+        <is>
+          <t>2026-08-18</t>
+        </is>
+      </c>
     </row>
     <row r="263">
       <c r="A263" t="inlineStr">
         <is>
-          <t>已确认</t>
+          <t>已实现</t>
         </is>
       </c>
       <c r="B263" t="inlineStr">
         <is>
-          <t>STEAM-DESKTOP-22G</t>
+          <t>STEAM-DESKTOP-08F</t>
         </is>
       </c>
       <c r="C263" t="inlineStr">
@@ -15240,7 +15232,7 @@
       </c>
       <c r="D263" t="inlineStr">
         <is>
-          <t>Overlay背景场景美术迭代</t>
+          <t>好友列表与申请 Prefab</t>
         </is>
       </c>
       <c r="E263" t="inlineStr">
@@ -15250,40 +15242,44 @@
       </c>
       <c r="F263" t="inlineStr">
         <is>
-          <t>后续迭代</t>
+          <t>v1.0-steam-desktop</t>
         </is>
       </c>
       <c r="G263" t="inlineStr">
         <is>
-          <t>P2</t>
+          <t>P0</t>
         </is>
       </c>
       <c r="H263" t="inlineStr">
         <is>
-          <t>仅记录：岸线、水面、钓位层次与风格优化，先预览后替换</t>
+          <t>独立 PanelFriends；修复接受/拒绝重叠不可点；不与 PanelSocial 双开好友 UI</t>
         </is>
       </c>
       <c r="I263" t="inlineStr">
         <is>
-          <t>docs/planning/specs/Steam桌面端-22鱼塘表现修复与后续迭代.md</t>
+          <t>docs/planning/specs/Steam桌面端-08F好友列表与申请Prefab.md</t>
         </is>
       </c>
       <c r="J263" t="inlineStr">
         <is>
-          <t>2026-10-24</t>
-        </is>
-      </c>
-      <c r="K263" t="inlineStr"/>
+          <t>2026-08-17</t>
+        </is>
+      </c>
+      <c r="K263" t="inlineStr">
+        <is>
+          <t>2026-08-17</t>
+        </is>
+      </c>
     </row>
     <row r="264">
       <c r="A264" t="inlineStr">
         <is>
-          <t>已确认</t>
+          <t>已实现</t>
         </is>
       </c>
       <c r="B264" t="inlineStr">
         <is>
-          <t>STEAM-DESKTOP-22H</t>
+          <t>STEAM-DESKTOP-08G</t>
         </is>
       </c>
       <c r="C264" t="inlineStr">
@@ -15293,7 +15289,7 @@
       </c>
       <c r="D264" t="inlineStr">
         <is>
-          <t>钓鱼过程特效</t>
+          <t>Overlay 钓鱼操作栏</t>
         </is>
       </c>
       <c r="E264" t="inlineStr">
@@ -15303,50 +15299,54 @@
       </c>
       <c r="F264" t="inlineStr">
         <is>
-          <t>后续迭代</t>
+          <t>v1.0-steam-desktop</t>
         </is>
       </c>
       <c r="G264" t="inlineStr">
         <is>
-          <t>P2</t>
+          <t>P0</t>
         </is>
       </c>
       <c r="H264" t="inlineStr">
         <is>
-          <t>仅记录：入水、波纹、咬钩、挣扎、收杆、脱钩反馈</t>
+          <t>Overlay 底部选钓位/开始/收杆/领鱼获；Pipe 发命令；Unity/Node 保留权威</t>
         </is>
       </c>
       <c r="I264" t="inlineStr">
         <is>
-          <t>docs/planning/specs/Steam桌面端-22鱼塘表现修复与后续迭代.md</t>
+          <t>docs/planning/specs/Steam桌面端-08GOverlay钓鱼操作栏.md</t>
         </is>
       </c>
       <c r="J264" t="inlineStr">
         <is>
-          <t>2026-10-24</t>
-        </is>
-      </c>
-      <c r="K264" t="inlineStr"/>
+          <t>2026-08-17</t>
+        </is>
+      </c>
+      <c r="K264" t="inlineStr">
+        <is>
+          <t>2026-08-17</t>
+        </is>
+      </c>
     </row>
     <row r="265">
       <c r="A265" t="inlineStr">
         <is>
-          <t>已确认</t>
+          <t>已实现</t>
         </is>
       </c>
       <c r="B265" t="inlineStr">
         <is>
-          <t>STEAM-DESKTOP-22I</t>
+          <t>STEAM-DESKTOP-08H</t>
         </is>
       </c>
       <c r="C265" t="inlineStr">
         <is>
-          <t>功能</t>
+          <t>工程</t>
         </is>
       </c>
       <c r="D265" t="inlineStr">
         <is>
-          <t>钓鱼与UI音效迭代</t>
+          <t>全量 UI 预制体化与动态内容组件</t>
         </is>
       </c>
       <c r="E265" t="inlineStr">
@@ -15356,50 +15356,54 @@
       </c>
       <c r="F265" t="inlineStr">
         <is>
-          <t>后续迭代</t>
+          <t>v1.0-steam-desktop</t>
         </is>
       </c>
       <c r="G265" t="inlineStr">
         <is>
-          <t>P2</t>
+          <t>P0</t>
         </is>
       </c>
       <c r="H265" t="inlineStr">
         <is>
-          <t>仅记录：音色、音量、触发时机与并发控制</t>
+          <t>壳层、功能页、列表行和 Grid item 全部使用合法 Prefab；运行时代码只绑定数据和事件</t>
         </is>
       </c>
       <c r="I265" t="inlineStr">
         <is>
-          <t>docs/planning/specs/Steam桌面端-22鱼塘表现修复与后续迭代.md</t>
+          <t>docs/planning/specs/Steam桌面端-08H全量UI预制体化.md</t>
         </is>
       </c>
       <c r="J265" t="inlineStr">
         <is>
-          <t>2026-10-24</t>
-        </is>
-      </c>
-      <c r="K265" t="inlineStr"/>
+          <t>2026-08-17</t>
+        </is>
+      </c>
+      <c r="K265" t="inlineStr">
+        <is>
+          <t>2026-08-17</t>
+        </is>
+      </c>
     </row>
     <row r="266">
       <c r="A266" t="inlineStr">
         <is>
-          <t>已确认</t>
+          <t>已实现</t>
         </is>
       </c>
       <c r="B266" t="inlineStr">
         <is>
-          <t>STEAM-DESKTOP-22J</t>
+          <t>STEAM-DESKTOP-08I</t>
         </is>
       </c>
       <c r="C266" t="inlineStr">
         <is>
-          <t>功能</t>
+          <t>Bug修复</t>
         </is>
       </c>
       <c r="D266" t="inlineStr">
         <is>
-          <t>世界地图迭代</t>
+          <t>鱼塘退出与跨塘切换优化</t>
         </is>
       </c>
       <c r="E266" t="inlineStr">
@@ -15409,30 +15413,34 @@
       </c>
       <c r="F266" t="inlineStr">
         <is>
-          <t>后续迭代</t>
+          <t>v1.0-steam-desktop</t>
         </is>
       </c>
       <c r="G266" t="inlineStr">
         <is>
-          <t>P2</t>
+          <t>P0</t>
         </is>
       </c>
       <c r="H266" t="inlineStr">
         <is>
-          <t>仅记录：信息层级、标识、筛选详情与进入路径；先交互预览</t>
+          <t>Overlay 点击钓位直接入座；新增离席/退出鱼塘；收杆领鱼离席后跨塘切换；修复隐藏主窗口时 5 FPS 导致的 ACK 延迟，增加 ACK 优先队列、持久状态序号、重复状态丢弃及三段链路时间戳验收</t>
         </is>
       </c>
       <c r="I266" t="inlineStr">
         <is>
-          <t>docs/planning/specs/Steam桌面端-22鱼塘表现修复与后续迭代.md</t>
+          <t>docs/planning/specs/Steam桌面端-08I鱼塘退出与跨塘切换优化.md</t>
         </is>
       </c>
       <c r="J266" t="inlineStr">
         <is>
-          <t>2026-10-24</t>
-        </is>
-      </c>
-      <c r="K266" t="inlineStr"/>
+          <t>2026-08-18</t>
+        </is>
+      </c>
+      <c r="K266" t="inlineStr">
+        <is>
+          <t>2026-08-18</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <autoFilter ref="A1:L135"/>

</xml_diff>

<commit_message>
## 2026-10-24 STEAM-DESKTOP-22K／22L／22M 呼吸、瞌睡与丧彪。STEAM-DESKTOP-22H／22I／22J 方案设计完善
</commit_message>
<xml_diff>
--- a/docs/planning/项目开发需求计划表.xlsx
+++ b/docs/planning/项目开发需求计划表.xlsx
@@ -454,7 +454,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L266"/>
+  <dimension ref="A1:L269"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -14412,12 +14412,12 @@
       </c>
       <c r="H248" t="inlineStr">
         <is>
-          <t>仅记录：入水、波纹、咬钩、挣扎、收杆、脱钩反馈</t>
+          <t>9类特效方案v1：共用事件/水面锚点、标准/简化/关闭、多人对象预算与验收；待视觉评审，未实现</t>
         </is>
       </c>
       <c r="I248" t="inlineStr">
         <is>
-          <t>docs/planning/specs/Steam桌面端-22鱼塘表现修复与后续迭代.md</t>
+          <t>docs/planning/specs/Steam桌面端-22H钓鱼特效设计.md</t>
         </is>
       </c>
       <c r="J248" t="inlineStr">
@@ -14464,12 +14464,12 @@
       </c>
       <c r="H249" t="inlineStr">
         <is>
-          <t>已制作6场景交互试听与4种候选音色；事件去重、加载同步、音量和并发方案待确认后接入</t>
+          <t>声音方案v1：沿用6场景试听，补齐事件去重、真实帧同步、声部/后台提示/资源规范；待听感评审，未接入</t>
         </is>
       </c>
       <c r="I249" t="inlineStr">
         <is>
-          <t>docs/planning/specs/Steam桌面端-22鱼塘表现修复与后续迭代.md</t>
+          <t>docs/planning/specs/Steam桌面端-22I声音体验设计.md</t>
         </is>
       </c>
       <c r="J249" t="inlineStr">
@@ -14516,12 +14516,12 @@
       </c>
       <c r="H250" t="inlineStr">
         <is>
-          <t>仅记录：信息层级、标识、筛选详情与进入路径；先交互预览</t>
+          <t>地图方案v1：三栏尺寸、真实点位/标签避让、筛选/缩放、档位费用确认与异常恢复；待交互评审，未实现</t>
         </is>
       </c>
       <c r="I250" t="inlineStr">
         <is>
-          <t>docs/planning/specs/Steam桌面端-22鱼塘表现修复与后续迭代.md</t>
+          <t>docs/planning/specs/Steam桌面端-22J世界地图设计.md</t>
         </is>
       </c>
       <c r="J250" t="inlineStr">
@@ -14538,7 +14538,7 @@
       </c>
       <c r="B251" t="inlineStr">
         <is>
-          <t>STEAM-DESKTOP-07A</t>
+          <t>STEAM-DESKTOP-22K</t>
         </is>
       </c>
       <c r="C251" t="inlineStr">
@@ -14548,7 +14548,7 @@
       </c>
       <c r="D251" t="inlineStr">
         <is>
-          <t>桌面宠物主视图与鱼塘入口</t>
+          <t>持续钓鱼呼吸</t>
         </is>
       </c>
       <c r="E251" t="inlineStr">
@@ -14558,32 +14558,32 @@
       </c>
       <c r="F251" t="inlineStr">
         <is>
-          <t>v1.0-steam-desktop</t>
+          <t>后续迭代</t>
         </is>
       </c>
       <c r="G251" t="inlineStr">
         <is>
-          <t>P0</t>
+          <t>P2</t>
         </is>
       </c>
       <c r="H251" t="inlineStr">
         <is>
-          <t>显示自己的 2D 猫咪、钓鱼状态和鱼塘入口；采用序列帧+状态机，复用已完成桌面壳</t>
+          <t>Unity/Overlay固定脚底有界呼吸、握竿同步及鱼线端点；Unity相关203/203、运动24/24；Windows待验收</t>
         </is>
       </c>
       <c r="I251" t="inlineStr">
         <is>
-          <t>docs/planning/specs/Steam桌面宠物与多人鱼塘表现层.md</t>
+          <t>docs/planning/specs/Steam桌面端-22KLM呼吸瞌睡与狸花猫.md</t>
         </is>
       </c>
       <c r="J251" t="inlineStr">
         <is>
-          <t>2026-08-13</t>
+          <t>2026-10-24</t>
         </is>
       </c>
       <c r="K251" t="inlineStr">
         <is>
-          <t>2026-08-14</t>
+          <t>2026-10-24</t>
         </is>
       </c>
     </row>
@@ -14595,7 +14595,7 @@
       </c>
       <c r="B252" t="inlineStr">
         <is>
-          <t>STEAM-DESKTOP-07B</t>
+          <t>STEAM-DESKTOP-22L</t>
         </is>
       </c>
       <c r="C252" t="inlineStr">
@@ -14605,7 +14605,7 @@
       </c>
       <c r="D252" t="inlineStr">
         <is>
-          <t>2D 鱼塘环境与自己的猫咪</t>
+          <t>挂机瞌睡与触碰唤醒</t>
         </is>
       </c>
       <c r="E252" t="inlineStr">
@@ -14615,32 +14615,32 @@
       </c>
       <c r="F252" t="inlineStr">
         <is>
-          <t>v1.0-steam-desktop</t>
+          <t>后续迭代</t>
         </is>
       </c>
       <c r="G252" t="inlineStr">
         <is>
-          <t>P0</t>
+          <t>P1</t>
         </is>
       </c>
       <c r="H252" t="inlineStr">
         <is>
-          <t>显示池塘环境、钓位、自己的宠物和钓鱼表现</t>
+          <t>默认30分钟，可配置；服务器持久化/直接逃鱼、本人触碰唤醒、11角色局部闭眼；服务端35/35；Windows待验收</t>
         </is>
       </c>
       <c r="I252" t="inlineStr">
         <is>
-          <t>docs/planning/specs/Steam桌面宠物与多人鱼塘表现层.md</t>
+          <t>docs/planning/specs/Steam桌面端-22KLM呼吸瞌睡与狸花猫.md</t>
         </is>
       </c>
       <c r="J252" t="inlineStr">
         <is>
-          <t>2026-08-13</t>
+          <t>2026-10-24</t>
         </is>
       </c>
       <c r="K252" t="inlineStr">
         <is>
-          <t>2026-08-14</t>
+          <t>2026-10-24</t>
         </is>
       </c>
     </row>
@@ -14652,17 +14652,17 @@
       </c>
       <c r="B253" t="inlineStr">
         <is>
-          <t>STEAM-DESKTOP-07C</t>
+          <t>STEAM-DESKTOP-22M</t>
         </is>
       </c>
       <c r="C253" t="inlineStr">
         <is>
-          <t>功能</t>
+          <t>美术</t>
         </is>
       </c>
       <c r="D253" t="inlineStr">
         <is>
-          <t>同塘玩家宠物与状态同步</t>
+          <t>狸花猫丧彪完整钓鱼动作</t>
         </is>
       </c>
       <c r="E253" t="inlineStr">
@@ -14672,32 +14672,32 @@
       </c>
       <c r="F253" t="inlineStr">
         <is>
-          <t>v1.0-steam-desktop</t>
+          <t>后续迭代</t>
         </is>
       </c>
       <c r="G253" t="inlineStr">
         <is>
-          <t>P0</t>
+          <t>P2</t>
         </is>
       </c>
       <c r="H253" t="inlineStr">
         <is>
-          <t>在 Overlay 渲染 pond_user_joined/left/updated；128×128 统一序列帧；fishingPhase→petVisualState；IPC 不传图、不新开协议</t>
+          <t>44原画/63源姿势/16钓鱼动作/74帧槽，头像与选择入口；家园仅站坐，未含行走进食翻滚蜷睡；Windows美术待验收</t>
         </is>
       </c>
       <c r="I253" t="inlineStr">
         <is>
-          <t>docs/planning/specs/Steam桌面宠物与多人鱼塘表现层.md</t>
+          <t>docs/planning/specs/Steam桌面端-22KLM呼吸瞌睡与狸花猫.md</t>
         </is>
       </c>
       <c r="J253" t="inlineStr">
         <is>
-          <t>2026-08-13</t>
+          <t>2026-10-24</t>
         </is>
       </c>
       <c r="K253" t="inlineStr">
         <is>
-          <t>2026-08-15</t>
+          <t>2026-10-24</t>
         </is>
       </c>
     </row>
@@ -14709,7 +14709,7 @@
       </c>
       <c r="B254" t="inlineStr">
         <is>
-          <t>STEAM-DESKTOP-07D</t>
+          <t>STEAM-DESKTOP-07A</t>
         </is>
       </c>
       <c r="C254" t="inlineStr">
@@ -14719,7 +14719,7 @@
       </c>
       <c r="D254" t="inlineStr">
         <is>
-          <t>桌面宠物右键菜单</t>
+          <t>桌面宠物主视图与鱼塘入口</t>
         </is>
       </c>
       <c r="E254" t="inlineStr">
@@ -14739,7 +14739,7 @@
       </c>
       <c r="H254" t="inlineStr">
         <is>
-          <t>在产品窗口/宠物区域提供鱼塘、好友、背包、图鉴、设置、托盘和退出入口</t>
+          <t>显示自己的 2D 猫咪、钓鱼状态和鱼塘入口；采用序列帧+状态机，复用已完成桌面壳</t>
         </is>
       </c>
       <c r="I254" t="inlineStr">
@@ -14754,7 +14754,7 @@
       </c>
       <c r="K254" t="inlineStr">
         <is>
-          <t>2026-08-16</t>
+          <t>2026-08-14</t>
         </is>
       </c>
     </row>
@@ -14766,7 +14766,7 @@
       </c>
       <c r="B255" t="inlineStr">
         <is>
-          <t>STEAM-DESKTOP-07E</t>
+          <t>STEAM-DESKTOP-07B</t>
         </is>
       </c>
       <c r="C255" t="inlineStr">
@@ -14776,7 +14776,7 @@
       </c>
       <c r="D255" t="inlineStr">
         <is>
-          <t>桌面宠物主窗口功能页签</t>
+          <t>2D 鱼塘环境与自己的猫咪</t>
         </is>
       </c>
       <c r="E255" t="inlineStr">
@@ -14796,12 +14796,12 @@
       </c>
       <c r="H255" t="inlineStr">
         <is>
-          <t>好友/聊天、背包、图鉴、设置为主窗口页签；Overlay 菜单切页且主窗口高于 Overlay；不用功能弹窗</t>
+          <t>显示池塘环境、钓位、自己的宠物和钓鱼表现</t>
         </is>
       </c>
       <c r="I255" t="inlineStr">
         <is>
-          <t>docs/planning/specs/Steam桌面端Web功能对齐设计.md</t>
+          <t>docs/planning/specs/Steam桌面宠物与多人鱼塘表现层.md</t>
         </is>
       </c>
       <c r="J255" t="inlineStr">
@@ -14811,7 +14811,7 @@
       </c>
       <c r="K255" t="inlineStr">
         <is>
-          <t>2026-08-17</t>
+          <t>2026-08-14</t>
         </is>
       </c>
     </row>
@@ -14823,7 +14823,7 @@
       </c>
       <c r="B256" t="inlineStr">
         <is>
-          <t>STEAM-DESKTOP-07F</t>
+          <t>STEAM-DESKTOP-07C</t>
         </is>
       </c>
       <c r="C256" t="inlineStr">
@@ -14833,7 +14833,7 @@
       </c>
       <c r="D256" t="inlineStr">
         <is>
-          <t>桌面宠物主流程与恢复验收</t>
+          <t>同塘玩家宠物与状态同步</t>
         </is>
       </c>
       <c r="E256" t="inlineStr">
@@ -14853,7 +14853,7 @@
       </c>
       <c r="H256" t="inlineStr">
         <is>
-          <t>串联登录、进塘、挂机、通知、托盘、收鱼、断线恢复并完成 Windows 验收</t>
+          <t>在 Overlay 渲染 pond_user_joined/left/updated；128×128 统一序列帧；fishingPhase→petVisualState；IPC 不传图、不新开协议</t>
         </is>
       </c>
       <c r="I256" t="inlineStr">
@@ -14868,7 +14868,7 @@
       </c>
       <c r="K256" t="inlineStr">
         <is>
-          <t>2026-08-17</t>
+          <t>2026-08-15</t>
         </is>
       </c>
     </row>
@@ -14880,7 +14880,7 @@
       </c>
       <c r="B257" t="inlineStr">
         <is>
-          <t>STEAM-DESKTOP-07G</t>
+          <t>STEAM-DESKTOP-07D</t>
         </is>
       </c>
       <c r="C257" t="inlineStr">
@@ -14890,7 +14890,7 @@
       </c>
       <c r="D257" t="inlineStr">
         <is>
-          <t>原生桌面宠物 Overlay</t>
+          <t>桌面宠物右键菜单</t>
         </is>
       </c>
       <c r="E257" t="inlineStr">
@@ -14905,27 +14905,27 @@
       </c>
       <c r="G257" t="inlineStr">
         <is>
-          <t>P1</t>
+          <t>P0</t>
         </is>
       </c>
       <c r="H257" t="inlineStr">
         <is>
-          <t>独立 WPF/Win32 Overlay；不启动第二个 Unity Player；通过 Named Pipe 接收状态并发送命令</t>
+          <t>在产品窗口/宠物区域提供鱼塘、好友、背包、图鉴、设置、托盘和退出入口</t>
         </is>
       </c>
       <c r="I257" t="inlineStr">
         <is>
-          <t>docs/planning/specs/Steam原生桌面宠物Overlay.md</t>
+          <t>docs/planning/specs/Steam桌面宠物与多人鱼塘表现层.md</t>
         </is>
       </c>
       <c r="J257" t="inlineStr">
         <is>
-          <t>2026-08-14</t>
+          <t>2026-08-13</t>
         </is>
       </c>
       <c r="K257" t="inlineStr">
         <is>
-          <t>2026-08-17</t>
+          <t>2026-08-16</t>
         </is>
       </c>
     </row>
@@ -14937,7 +14937,7 @@
       </c>
       <c r="B258" t="inlineStr">
         <is>
-          <t>STEAM-DESKTOP-08A</t>
+          <t>STEAM-DESKTOP-07E</t>
         </is>
       </c>
       <c r="C258" t="inlineStr">
@@ -14947,7 +14947,7 @@
       </c>
       <c r="D258" t="inlineStr">
         <is>
-          <t>世界地图与鱼塘选择</t>
+          <t>桌面宠物主窗口功能页签</t>
         </is>
       </c>
       <c r="E258" t="inlineStr">
@@ -14967,17 +14967,17 @@
       </c>
       <c r="H258" t="inlineStr">
         <is>
-          <t>主窗口超大地图 Image：拖动/滚轮缩放/边界；pondId 坐标绑定；点击进塘并显示 Overlay</t>
+          <t>好友/聊天、背包、图鉴、设置为主窗口页签；Overlay 菜单切页且主窗口高于 Overlay；不用功能弹窗</t>
         </is>
       </c>
       <c r="I258" t="inlineStr">
         <is>
-          <t>docs/planning/specs/Steam桌面端-08A世界地图与鱼塘选择.md</t>
+          <t>docs/planning/specs/Steam桌面端Web功能对齐设计.md</t>
         </is>
       </c>
       <c r="J258" t="inlineStr">
         <is>
-          <t>2026-08-17</t>
+          <t>2026-08-13</t>
         </is>
       </c>
       <c r="K258" t="inlineStr">
@@ -14994,7 +14994,7 @@
       </c>
       <c r="B259" t="inlineStr">
         <is>
-          <t>STEAM-DESKTOP-08B</t>
+          <t>STEAM-DESKTOP-07F</t>
         </is>
       </c>
       <c r="C259" t="inlineStr">
@@ -15004,7 +15004,7 @@
       </c>
       <c r="D259" t="inlineStr">
         <is>
-          <t>商店与装备</t>
+          <t>桌面宠物主流程与恢复验收</t>
         </is>
       </c>
       <c r="E259" t="inlineStr">
@@ -15024,22 +15024,22 @@
       </c>
       <c r="H259" t="inlineStr">
         <is>
-          <t>PanelShop：鱼饵/渔具购买与装备；金币库存以服务端为准；Overlay 只 menu_shop 切页</t>
+          <t>串联登录、进塘、挂机、通知、托盘、收鱼、断线恢复并完成 Windows 验收</t>
         </is>
       </c>
       <c r="I259" t="inlineStr">
         <is>
-          <t>docs/planning/specs/Steam桌面端-08B商店与装备.md</t>
+          <t>docs/planning/specs/Steam桌面宠物与多人鱼塘表现层.md</t>
         </is>
       </c>
       <c r="J259" t="inlineStr">
         <is>
+          <t>2026-08-13</t>
+        </is>
+      </c>
+      <c r="K259" t="inlineStr">
+        <is>
           <t>2026-08-17</t>
-        </is>
-      </c>
-      <c r="K259" t="inlineStr">
-        <is>
-          <t>2026-08-18</t>
         </is>
       </c>
     </row>
@@ -15051,7 +15051,7 @@
       </c>
       <c r="B260" t="inlineStr">
         <is>
-          <t>STEAM-DESKTOP-08C</t>
+          <t>STEAM-DESKTOP-07G</t>
         </is>
       </c>
       <c r="C260" t="inlineStr">
@@ -15061,7 +15061,7 @@
       </c>
       <c r="D260" t="inlineStr">
         <is>
-          <t>动态墙与好友动态</t>
+          <t>原生桌面宠物 Overlay</t>
         </is>
       </c>
       <c r="E260" t="inlineStr">
@@ -15081,22 +15081,22 @@
       </c>
       <c r="H260" t="inlineStr">
         <is>
-          <t>PanelSocialFeed：公共/好友动态、分页加载、动态卡片 Prefab、点赞、评论、删除评论；不塞进 PanelSocial</t>
+          <t>独立 WPF/Win32 Overlay；不启动第二个 Unity Player；通过 Named Pipe 接收状态并发送命令</t>
         </is>
       </c>
       <c r="I260" t="inlineStr">
         <is>
-          <t>docs/planning/specs/Steam桌面端-08C动态墙与好友动态.md</t>
+          <t>docs/planning/specs/Steam原生桌面宠物Overlay.md</t>
         </is>
       </c>
       <c r="J260" t="inlineStr">
         <is>
+          <t>2026-08-14</t>
+        </is>
+      </c>
+      <c r="K260" t="inlineStr">
+        <is>
           <t>2026-08-17</t>
-        </is>
-      </c>
-      <c r="K260" t="inlineStr">
-        <is>
-          <t>2026-08-19</t>
         </is>
       </c>
     </row>
@@ -15108,7 +15108,7 @@
       </c>
       <c r="B261" t="inlineStr">
         <is>
-          <t>STEAM-DESKTOP-08D</t>
+          <t>STEAM-DESKTOP-08A</t>
         </is>
       </c>
       <c r="C261" t="inlineStr">
@@ -15118,7 +15118,7 @@
       </c>
       <c r="D261" t="inlineStr">
         <is>
-          <t>排行榜</t>
+          <t>世界地图与鱼塘选择</t>
         </is>
       </c>
       <c r="E261" t="inlineStr">
@@ -15133,17 +15133,17 @@
       </c>
       <c r="G261" t="inlineStr">
         <is>
-          <t>P1</t>
+          <t>P0</t>
         </is>
       </c>
       <c r="H261" t="inlineStr">
         <is>
-          <t>PanelLeaderboard：日/周/鱼塘/稀有四榜；Top3 固定 Image 领奖台；4 名起纵向滚动；分数以服务端为准</t>
+          <t>主窗口超大地图 Image：拖动/滚轮缩放/边界；pondId 坐标绑定；点击进塘并显示 Overlay</t>
         </is>
       </c>
       <c r="I261" t="inlineStr">
         <is>
-          <t>docs/planning/specs/Steam桌面端-08D排行榜.md</t>
+          <t>docs/planning/specs/Steam桌面端-08A世界地图与鱼塘选择.md</t>
         </is>
       </c>
       <c r="J261" t="inlineStr">
@@ -15153,7 +15153,7 @@
       </c>
       <c r="K261" t="inlineStr">
         <is>
-          <t>2026-08-20</t>
+          <t>2026-08-17</t>
         </is>
       </c>
     </row>
@@ -15165,7 +15165,7 @@
       </c>
       <c r="B262" t="inlineStr">
         <is>
-          <t>STEAM-DESKTOP-08E</t>
+          <t>STEAM-DESKTOP-08B</t>
         </is>
       </c>
       <c r="C262" t="inlineStr">
@@ -15175,7 +15175,7 @@
       </c>
       <c r="D262" t="inlineStr">
         <is>
-          <t>个人中心与资料编辑</t>
+          <t>商店与装备</t>
         </is>
       </c>
       <c r="E262" t="inlineStr">
@@ -15190,17 +15190,17 @@
       </c>
       <c r="G262" t="inlineStr">
         <is>
-          <t>P1</t>
+          <t>P0</t>
         </is>
       </c>
       <c r="H262" t="inlineStr">
         <is>
-          <t>PanelProfile/Edit：昵称头像展示鱼获；不改 SteamID、不迁移旧档</t>
+          <t>PanelShop：鱼饵/渔具购买与装备；金币库存以服务端为准；Overlay 只 menu_shop 切页</t>
         </is>
       </c>
       <c r="I262" t="inlineStr">
         <is>
-          <t>docs/planning/specs/Steam桌面端-08E个人中心与资料编辑.md</t>
+          <t>docs/planning/specs/Steam桌面端-08B商店与装备.md</t>
         </is>
       </c>
       <c r="J262" t="inlineStr">
@@ -15222,7 +15222,7 @@
       </c>
       <c r="B263" t="inlineStr">
         <is>
-          <t>STEAM-DESKTOP-08F</t>
+          <t>STEAM-DESKTOP-08C</t>
         </is>
       </c>
       <c r="C263" t="inlineStr">
@@ -15232,7 +15232,7 @@
       </c>
       <c r="D263" t="inlineStr">
         <is>
-          <t>好友列表与申请 Prefab</t>
+          <t>动态墙与好友动态</t>
         </is>
       </c>
       <c r="E263" t="inlineStr">
@@ -15247,17 +15247,17 @@
       </c>
       <c r="G263" t="inlineStr">
         <is>
-          <t>P0</t>
+          <t>P1</t>
         </is>
       </c>
       <c r="H263" t="inlineStr">
         <is>
-          <t>独立 PanelFriends；修复接受/拒绝重叠不可点；不与 PanelSocial 双开好友 UI</t>
+          <t>PanelSocialFeed：公共/好友动态、分页加载、动态卡片 Prefab、点赞、评论、删除评论；不塞进 PanelSocial</t>
         </is>
       </c>
       <c r="I263" t="inlineStr">
         <is>
-          <t>docs/planning/specs/Steam桌面端-08F好友列表与申请Prefab.md</t>
+          <t>docs/planning/specs/Steam桌面端-08C动态墙与好友动态.md</t>
         </is>
       </c>
       <c r="J263" t="inlineStr">
@@ -15267,7 +15267,7 @@
       </c>
       <c r="K263" t="inlineStr">
         <is>
-          <t>2026-08-17</t>
+          <t>2026-08-19</t>
         </is>
       </c>
     </row>
@@ -15279,7 +15279,7 @@
       </c>
       <c r="B264" t="inlineStr">
         <is>
-          <t>STEAM-DESKTOP-08G</t>
+          <t>STEAM-DESKTOP-08D</t>
         </is>
       </c>
       <c r="C264" t="inlineStr">
@@ -15289,7 +15289,7 @@
       </c>
       <c r="D264" t="inlineStr">
         <is>
-          <t>Overlay 钓鱼操作栏</t>
+          <t>排行榜</t>
         </is>
       </c>
       <c r="E264" t="inlineStr">
@@ -15304,17 +15304,17 @@
       </c>
       <c r="G264" t="inlineStr">
         <is>
-          <t>P0</t>
+          <t>P1</t>
         </is>
       </c>
       <c r="H264" t="inlineStr">
         <is>
-          <t>Overlay 底部选钓位/开始/收杆/领鱼获；Pipe 发命令；Unity/Node 保留权威</t>
+          <t>PanelLeaderboard：日/周/鱼塘/稀有四榜；Top3 固定 Image 领奖台；4 名起纵向滚动；分数以服务端为准</t>
         </is>
       </c>
       <c r="I264" t="inlineStr">
         <is>
-          <t>docs/planning/specs/Steam桌面端-08GOverlay钓鱼操作栏.md</t>
+          <t>docs/planning/specs/Steam桌面端-08D排行榜.md</t>
         </is>
       </c>
       <c r="J264" t="inlineStr">
@@ -15324,7 +15324,7 @@
       </c>
       <c r="K264" t="inlineStr">
         <is>
-          <t>2026-08-17</t>
+          <t>2026-08-20</t>
         </is>
       </c>
     </row>
@@ -15336,17 +15336,17 @@
       </c>
       <c r="B265" t="inlineStr">
         <is>
-          <t>STEAM-DESKTOP-08H</t>
+          <t>STEAM-DESKTOP-08E</t>
         </is>
       </c>
       <c r="C265" t="inlineStr">
         <is>
-          <t>工程</t>
+          <t>功能</t>
         </is>
       </c>
       <c r="D265" t="inlineStr">
         <is>
-          <t>全量 UI 预制体化与动态内容组件</t>
+          <t>个人中心与资料编辑</t>
         </is>
       </c>
       <c r="E265" t="inlineStr">
@@ -15361,17 +15361,17 @@
       </c>
       <c r="G265" t="inlineStr">
         <is>
-          <t>P0</t>
+          <t>P1</t>
         </is>
       </c>
       <c r="H265" t="inlineStr">
         <is>
-          <t>壳层、功能页、列表行和 Grid item 全部使用合法 Prefab；运行时代码只绑定数据和事件</t>
+          <t>PanelProfile/Edit：昵称头像展示鱼获；不改 SteamID、不迁移旧档</t>
         </is>
       </c>
       <c r="I265" t="inlineStr">
         <is>
-          <t>docs/planning/specs/Steam桌面端-08H全量UI预制体化.md</t>
+          <t>docs/planning/specs/Steam桌面端-08E个人中心与资料编辑.md</t>
         </is>
       </c>
       <c r="J265" t="inlineStr">
@@ -15381,7 +15381,7 @@
       </c>
       <c r="K265" t="inlineStr">
         <is>
-          <t>2026-08-17</t>
+          <t>2026-08-18</t>
         </is>
       </c>
     </row>
@@ -15393,50 +15393,221 @@
       </c>
       <c r="B266" t="inlineStr">
         <is>
+          <t>STEAM-DESKTOP-08F</t>
+        </is>
+      </c>
+      <c r="C266" t="inlineStr">
+        <is>
+          <t>功能</t>
+        </is>
+      </c>
+      <c r="D266" t="inlineStr">
+        <is>
+          <t>好友列表与申请 Prefab</t>
+        </is>
+      </c>
+      <c r="E266" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F266" t="inlineStr">
+        <is>
+          <t>v1.0-steam-desktop</t>
+        </is>
+      </c>
+      <c r="G266" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="H266" t="inlineStr">
+        <is>
+          <t>独立 PanelFriends；修复接受/拒绝重叠不可点；不与 PanelSocial 双开好友 UI</t>
+        </is>
+      </c>
+      <c r="I266" t="inlineStr">
+        <is>
+          <t>docs/planning/specs/Steam桌面端-08F好友列表与申请Prefab.md</t>
+        </is>
+      </c>
+      <c r="J266" t="inlineStr">
+        <is>
+          <t>2026-08-17</t>
+        </is>
+      </c>
+      <c r="K266" t="inlineStr">
+        <is>
+          <t>2026-08-17</t>
+        </is>
+      </c>
+    </row>
+    <row r="267">
+      <c r="A267" t="inlineStr">
+        <is>
+          <t>已实现</t>
+        </is>
+      </c>
+      <c r="B267" t="inlineStr">
+        <is>
+          <t>STEAM-DESKTOP-08G</t>
+        </is>
+      </c>
+      <c r="C267" t="inlineStr">
+        <is>
+          <t>功能</t>
+        </is>
+      </c>
+      <c r="D267" t="inlineStr">
+        <is>
+          <t>Overlay 钓鱼操作栏</t>
+        </is>
+      </c>
+      <c r="E267" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F267" t="inlineStr">
+        <is>
+          <t>v1.0-steam-desktop</t>
+        </is>
+      </c>
+      <c r="G267" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="H267" t="inlineStr">
+        <is>
+          <t>Overlay 底部选钓位/开始/收杆/领鱼获；Pipe 发命令；Unity/Node 保留权威</t>
+        </is>
+      </c>
+      <c r="I267" t="inlineStr">
+        <is>
+          <t>docs/planning/specs/Steam桌面端-08GOverlay钓鱼操作栏.md</t>
+        </is>
+      </c>
+      <c r="J267" t="inlineStr">
+        <is>
+          <t>2026-08-17</t>
+        </is>
+      </c>
+      <c r="K267" t="inlineStr">
+        <is>
+          <t>2026-08-17</t>
+        </is>
+      </c>
+    </row>
+    <row r="268">
+      <c r="A268" t="inlineStr">
+        <is>
+          <t>已实现</t>
+        </is>
+      </c>
+      <c r="B268" t="inlineStr">
+        <is>
+          <t>STEAM-DESKTOP-08H</t>
+        </is>
+      </c>
+      <c r="C268" t="inlineStr">
+        <is>
+          <t>工程</t>
+        </is>
+      </c>
+      <c r="D268" t="inlineStr">
+        <is>
+          <t>全量 UI 预制体化与动态内容组件</t>
+        </is>
+      </c>
+      <c r="E268" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F268" t="inlineStr">
+        <is>
+          <t>v1.0-steam-desktop</t>
+        </is>
+      </c>
+      <c r="G268" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="H268" t="inlineStr">
+        <is>
+          <t>壳层、功能页、列表行和 Grid item 全部使用合法 Prefab；运行时代码只绑定数据和事件</t>
+        </is>
+      </c>
+      <c r="I268" t="inlineStr">
+        <is>
+          <t>docs/planning/specs/Steam桌面端-08H全量UI预制体化.md</t>
+        </is>
+      </c>
+      <c r="J268" t="inlineStr">
+        <is>
+          <t>2026-08-17</t>
+        </is>
+      </c>
+      <c r="K268" t="inlineStr">
+        <is>
+          <t>2026-08-17</t>
+        </is>
+      </c>
+    </row>
+    <row r="269">
+      <c r="A269" t="inlineStr">
+        <is>
+          <t>已实现</t>
+        </is>
+      </c>
+      <c r="B269" t="inlineStr">
+        <is>
           <t>STEAM-DESKTOP-08I</t>
         </is>
       </c>
-      <c r="C266" t="inlineStr">
+      <c r="C269" t="inlineStr">
         <is>
           <t>Bug修复</t>
         </is>
       </c>
-      <c r="D266" t="inlineStr">
+      <c r="D269" t="inlineStr">
         <is>
           <t>鱼塘退出与跨塘切换优化</t>
         </is>
       </c>
-      <c r="E266" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="F266" t="inlineStr">
+      <c r="E269" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F269" t="inlineStr">
         <is>
           <t>v1.0-steam-desktop</t>
         </is>
       </c>
-      <c r="G266" t="inlineStr">
+      <c r="G269" t="inlineStr">
         <is>
           <t>P0</t>
         </is>
       </c>
-      <c r="H266" t="inlineStr">
+      <c r="H269" t="inlineStr">
         <is>
           <t>Overlay 点击钓位直接入座；新增离席/退出鱼塘；收杆领鱼离席后跨塘切换；修复隐藏主窗口时 5 FPS 导致的 ACK 延迟，增加 ACK 优先队列、持久状态序号、重复状态丢弃及三段链路时间戳验收</t>
         </is>
       </c>
-      <c r="I266" t="inlineStr">
+      <c r="I269" t="inlineStr">
         <is>
           <t>docs/planning/specs/Steam桌面端-08I鱼塘退出与跨塘切换优化.md</t>
         </is>
       </c>
-      <c r="J266" t="inlineStr">
+      <c r="J269" t="inlineStr">
         <is>
           <t>2026-08-18</t>
         </is>
       </c>
-      <c r="K266" t="inlineStr">
+      <c r="K269" t="inlineStr">
         <is>
           <t>2026-08-18</t>
         </is>

</xml_diff>

<commit_message>
## 2026-10-24 — STEAM-DESKTOP-22I v2 工程实现
</commit_message>
<xml_diff>
--- a/docs/planning/项目开发需求计划表.xlsx
+++ b/docs/planning/项目开发需求计划表.xlsx
@@ -14412,7 +14412,7 @@
       </c>
       <c r="H248" t="inlineStr">
         <is>
-          <t>9类特效方案v1：共用事件/水面锚点、标准/简化/关闭、多人对象预算与验收；待视觉评审，未实现</t>
+          <t>资源/代码已接入：四档18纹理、11角色预览、池化Overlay及Unity兜底；本机验证已执行；Windows/I联测与视觉验收待完成，完成日期暂留空</t>
         </is>
       </c>
       <c r="I248" t="inlineStr">
@@ -14429,7 +14429,7 @@
     <row r="249">
       <c r="A249" t="inlineStr">
         <is>
-          <t>已确认</t>
+          <t>已实现</t>
         </is>
       </c>
       <c r="B249" t="inlineStr">
@@ -14464,7 +14464,7 @@
       </c>
       <c r="H249" t="inlineStr">
         <is>
-          <t>声音方案v1：沿用6场景试听，补齐事件去重、真实帧同步、声部/后台提示/资源规范；待听感评审，未接入</t>
+          <t>v2纸张物音/28条独立实录水声/柔音钢琴循环/九场景A-B；Unity-WPF事件去重与四声部接入，工程验证通过；Windows画声延迟和耳机/扬声器听感待验收</t>
         </is>
       </c>
       <c r="I249" t="inlineStr">
@@ -14473,6 +14473,11 @@
         </is>
       </c>
       <c r="J249" t="inlineStr">
+        <is>
+          <t>2026-10-24</t>
+        </is>
+      </c>
+      <c r="K249" t="inlineStr">
         <is>
           <t>2026-10-24</t>
         </is>

</xml_diff>

<commit_message>
## 2026-10-24 — STEAM-DESKTOP-22I 当前方案采用与清理
</commit_message>
<xml_diff>
--- a/docs/planning/项目开发需求计划表.xlsx
+++ b/docs/planning/项目开发需求计划表.xlsx
@@ -14412,7 +14412,7 @@
       </c>
       <c r="H248" t="inlineStr">
         <is>
-          <t>资源/代码已接入：四档18纹理、11角色预览、池化Overlay及Unity兜底；本机验证已执行；Windows/I联测与视觉验收待完成，完成日期暂留空</t>
+          <t>v4风格已确认；按追加要求区分波纹/飞溅并修正入水落点，恢复真实收杆触水；Overlay/Unity本机验证，Windows/I实机待验收</t>
         </is>
       </c>
       <c r="I248" t="inlineStr">
@@ -14464,7 +14464,7 @@
       </c>
       <c r="H249" t="inlineStr">
         <is>
-          <t>v2纸张物音/28条独立实录水声/柔音钢琴循环/九场景A-B；Unity-WPF事件去重与四声部接入，工程验证通过；Windows画声延迟和耳机/扬声器听感待验收</t>
+          <t>v5配乐与46条v3音效及猫声已采用并应用；旧版音频和无效工具已清理，来源许可留档；Unity-WPF已接入，Windows画声延迟待实测</t>
         </is>
       </c>
       <c r="I249" t="inlineStr">

</xml_diff>

<commit_message>
## 2026-10-25 — STEAM-DESKTOP-22H 正式采用
</commit_message>
<xml_diff>
--- a/docs/planning/项目开发需求计划表.xlsx
+++ b/docs/planning/项目开发需求计划表.xlsx
@@ -14377,7 +14377,7 @@
     <row r="248">
       <c r="A248" t="inlineStr">
         <is>
-          <t>已确认</t>
+          <t>已实现</t>
         </is>
       </c>
       <c r="B248" t="inlineStr">
@@ -14412,7 +14412,7 @@
       </c>
       <c r="H248" t="inlineStr">
         <is>
-          <t>v4风格已确认；按追加要求区分波纹/飞溅并修正入水落点，恢复真实收杆触水；Overlay/Unity本机验证，Windows/I实机待验收</t>
+          <t>用户正式采用v4造型与v8鱼塘配色；七类真实触水效果、放大波纹及三端接入完成，本机验证通过；Windows性能/点击穿透及H/I实机待验收</t>
         </is>
       </c>
       <c r="I248" t="inlineStr">
@@ -14423,6 +14423,11 @@
       <c r="J248" t="inlineStr">
         <is>
           <t>2026-10-24</t>
+        </is>
+      </c>
+      <c r="K248" t="inlineStr">
+        <is>
+          <t>2026-10-25</t>
         </is>
       </c>
     </row>

</xml_diff>